<commit_message>
20260206 - Ajustes em telas, regras e navegação
</commit_message>
<xml_diff>
--- a/docs/Variáveis.xlsx
+++ b/docs/Variáveis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC01\OneDrive\Projetos\corrida-training-system\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E316EFB8-5322-43BA-98F1-82B894765968}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EEB86F1-F104-45FF-969E-595118B07A05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{CEA2BF3F-4FB1-457C-9393-73CD8B81DDE1}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="106">
   <si>
     <t>FC Máxima no Teste</t>
   </si>
@@ -276,6 +276,84 @@
   </si>
   <si>
     <t>Título</t>
+  </si>
+  <si>
+    <t>Aporte Energético</t>
+  </si>
+  <si>
+    <t>Estratégia de aporte energético</t>
+  </si>
+  <si>
+    <t>Diferença % em relação à necessidade estimada</t>
+  </si>
+  <si>
+    <t>Tipo de Dieta</t>
+  </si>
+  <si>
+    <t>Disponibilidade Energética</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aporte energético Diário Sugerido </t>
+  </si>
+  <si>
+    <t>Diferença Absoluta Necessidade vs Consumo</t>
+  </si>
+  <si>
+    <t>Diferença Percentual Necessidade vs Consumo</t>
+  </si>
+  <si>
+    <t>Macronutrientes</t>
+  </si>
+  <si>
+    <t>Total de Kcal/dia</t>
+  </si>
+  <si>
+    <t>Estimativa de Emagrecimento:</t>
+  </si>
+  <si>
+    <t>Variação de Redução de Gordura Estimada</t>
+  </si>
+  <si>
+    <t>Variação de Redução 1kg de gordura</t>
+  </si>
+  <si>
+    <t>Variação da meta proposta (-0,1kg)</t>
+  </si>
+  <si>
+    <t>Proteínas (g/kg)</t>
+  </si>
+  <si>
+    <t>Carboidratos (g/kg)</t>
+  </si>
+  <si>
+    <t>Lipídios (g/kg)</t>
+  </si>
+  <si>
+    <t>Proteínas (g/dia)</t>
+  </si>
+  <si>
+    <t>Carboidratos (g/dia)</t>
+  </si>
+  <si>
+    <t>Lipídios (g/dia)</t>
+  </si>
+  <si>
+    <t>Proteínas (kcal/dia)</t>
+  </si>
+  <si>
+    <t>Carboidratos (kcal/dia)</t>
+  </si>
+  <si>
+    <t>Lipídios (kcal/dia)</t>
+  </si>
+  <si>
+    <t>Proteínas (%)</t>
+  </si>
+  <si>
+    <t>Carboidratos (%)</t>
+  </si>
+  <si>
+    <t>Lipídios (%)</t>
   </si>
 </sst>
 </file>
@@ -311,8 +389,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -647,12 +728,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10F2A677-5D77-426F-B7DB-90429FF6A669}">
-  <dimension ref="A1:C68"/>
+  <dimension ref="A1:C90"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="33" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="26.625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="28.125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="68.875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1295,6 +1376,248 @@
         <v>0</v>
       </c>
     </row>
+    <row r="69" spans="1:3">
+      <c r="A69" t="s">
+        <v>80</v>
+      </c>
+      <c r="B69" t="s">
+        <v>81</v>
+      </c>
+      <c r="C69" s="1" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3">
+      <c r="A70" t="s">
+        <v>80</v>
+      </c>
+      <c r="B70" t="s">
+        <v>81</v>
+      </c>
+      <c r="C70" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3">
+      <c r="A71" t="s">
+        <v>80</v>
+      </c>
+      <c r="B71" t="s">
+        <v>81</v>
+      </c>
+      <c r="C71" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3">
+      <c r="A72" t="s">
+        <v>80</v>
+      </c>
+      <c r="B72" t="s">
+        <v>81</v>
+      </c>
+      <c r="C72" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3">
+      <c r="A73" t="s">
+        <v>80</v>
+      </c>
+      <c r="B73" t="s">
+        <v>81</v>
+      </c>
+      <c r="C73" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3">
+      <c r="A74" t="s">
+        <v>80</v>
+      </c>
+      <c r="B74" t="s">
+        <v>81</v>
+      </c>
+      <c r="C74" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3">
+      <c r="A75" t="s">
+        <v>80</v>
+      </c>
+      <c r="B75" t="s">
+        <v>88</v>
+      </c>
+      <c r="C75" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3">
+      <c r="A76" t="s">
+        <v>80</v>
+      </c>
+      <c r="B76" t="s">
+        <v>88</v>
+      </c>
+      <c r="C76" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3">
+      <c r="A77" t="s">
+        <v>80</v>
+      </c>
+      <c r="B77" t="s">
+        <v>88</v>
+      </c>
+      <c r="C77" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3">
+      <c r="A78" t="s">
+        <v>80</v>
+      </c>
+      <c r="B78" t="s">
+        <v>88</v>
+      </c>
+      <c r="C78" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3">
+      <c r="A79" t="s">
+        <v>80</v>
+      </c>
+      <c r="B79" t="s">
+        <v>88</v>
+      </c>
+      <c r="C79" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3">
+      <c r="A80" t="s">
+        <v>80</v>
+      </c>
+      <c r="B80" t="s">
+        <v>88</v>
+      </c>
+      <c r="C80" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3">
+      <c r="A81" t="s">
+        <v>80</v>
+      </c>
+      <c r="B81" t="s">
+        <v>88</v>
+      </c>
+      <c r="C81" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3">
+      <c r="A82" t="s">
+        <v>80</v>
+      </c>
+      <c r="B82" t="s">
+        <v>88</v>
+      </c>
+      <c r="C82" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3">
+      <c r="A83" t="s">
+        <v>80</v>
+      </c>
+      <c r="B83" t="s">
+        <v>88</v>
+      </c>
+      <c r="C83" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3">
+      <c r="A84" t="s">
+        <v>80</v>
+      </c>
+      <c r="B84" t="s">
+        <v>88</v>
+      </c>
+      <c r="C84" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3">
+      <c r="A85" t="s">
+        <v>80</v>
+      </c>
+      <c r="B85" t="s">
+        <v>88</v>
+      </c>
+      <c r="C85" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3">
+      <c r="A86" t="s">
+        <v>80</v>
+      </c>
+      <c r="B86" t="s">
+        <v>88</v>
+      </c>
+      <c r="C86" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3">
+      <c r="A87" t="s">
+        <v>80</v>
+      </c>
+      <c r="B87" t="s">
+        <v>88</v>
+      </c>
+      <c r="C87" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3">
+      <c r="A88" t="s">
+        <v>80</v>
+      </c>
+      <c r="B88" t="s">
+        <v>90</v>
+      </c>
+      <c r="C88" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3">
+      <c r="A89" t="s">
+        <v>80</v>
+      </c>
+      <c r="B89" t="s">
+        <v>90</v>
+      </c>
+      <c r="C89" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3">
+      <c r="A90" t="s">
+        <v>80</v>
+      </c>
+      <c r="B90" t="s">
+        <v>90</v>
+      </c>
+      <c r="C90" t="s">
+        <v>93</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
20260212 - Alteração da pasta e renomear do projeto para "training_system"
</commit_message>
<xml_diff>
--- a/docs/Variáveis.xlsx
+++ b/docs/Variáveis.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC01\OneDrive\Projetos\corrida-training-system\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EEB86F1-F104-45FF-969E-595118B07A05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F72D317C-2C7A-4D42-B153-AA5CD43C6B14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{CEA2BF3F-4FB1-457C-9393-73CD8B81DDE1}"/>
+    <workbookView xWindow="-1200" yWindow="3075" windowWidth="21600" windowHeight="11295" xr2:uid="{CEA2BF3F-4FB1-457C-9393-73CD8B81DDE1}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="110">
   <si>
     <t>FC Máxima no Teste</t>
   </si>
@@ -354,6 +354,18 @@
   </si>
   <si>
     <t>Lipídios (%)</t>
+  </si>
+  <si>
+    <t>ESCALA DE PERCEPÇÃO SUBJETIVA DE ESFORÇO (PSE)</t>
+  </si>
+  <si>
+    <t>ESCALA DE PERCEPÇÃO SUBJETIVA DE RECUPERAÇÃO (PSR)</t>
+  </si>
+  <si>
+    <t>Escala de Percepção</t>
+  </si>
+  <si>
+    <t>Perceção Subjetiva de Esforço (PSE)</t>
   </si>
 </sst>
 </file>
@@ -728,10 +740,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10F2A677-5D77-426F-B7DB-90429FF6A669}">
-  <dimension ref="A1:C90"/>
+  <dimension ref="A1:C94"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="33" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="45.75" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="26.625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="68.875" customWidth="1"/>
   </cols>
@@ -1618,6 +1630,24 @@
         <v>93</v>
       </c>
     </row>
+    <row r="91" spans="1:3">
+      <c r="A91" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3">
+      <c r="A92" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3">
+      <c r="A94" t="s">
+        <v>108</v>
+      </c>
+      <c r="B94" t="s">
+        <v>109</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>